<commit_message>
Updates fixed covid numbers
</commit_message>
<xml_diff>
--- a/apportion/pop.xlsx
+++ b/apportion/pop.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Google Drive/GitHub/R Functions/apportion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848E51B3-F7F6-BE46-931F-2DA7DCB26CA6}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A3C4D6-0D34-2043-B0CF-EBDF49C09E7B}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35840" yWindow="-6380" windowWidth="21600" windowHeight="37900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pop" sheetId="1" r:id="rId1"/>
@@ -421,9 +421,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -554,13 +554,6 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -909,14 +902,13 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1277,8 +1269,8 @@
   <dimension ref="A1:AA52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="26" max="26" width="17.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.83203125" style="6"/>
+    <col min="26" max="26" width="17.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.2">
@@ -1357,10 +1349,10 @@
       <c r="Y1" t="s">
         <v>124</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="Z1" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AA1" s="5" t="s">
         <v>128</v>
       </c>
     </row>
@@ -1369,7 +1361,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C2">
         <v>4802982</v>
@@ -1381,15 +1373,15 @@
         <v>4921532</v>
       </c>
       <c r="F2">
-        <f>D2-C2</f>
+        <f t="shared" ref="F2:F33" si="0">D2-C2</f>
         <v>227071</v>
       </c>
       <c r="G2">
-        <f>F2/C2*100</f>
+        <f t="shared" ref="G2:G33" si="1">F2/C2*100</f>
         <v>4.7277087442759518</v>
       </c>
       <c r="H2" s="2">
-        <f>(D2-E2)/E2</f>
+        <f t="shared" ref="H2:H33" si="2">(D2-E2)/E2</f>
         <v>2.2050247768377815E-2</v>
       </c>
       <c r="I2">
@@ -1399,37 +1391,37 @@
         <v>7</v>
       </c>
       <c r="K2">
-        <f>J2-I2</f>
+        <f t="shared" ref="K2:K33" si="3">J2-I2</f>
         <v>0</v>
       </c>
       <c r="L2">
         <v>9</v>
       </c>
       <c r="M2">
-        <f>J2+2</f>
+        <f t="shared" ref="M2:M9" si="4">J2+2</f>
         <v>9</v>
       </c>
       <c r="N2">
-        <f>M2-L2</f>
+        <f t="shared" ref="N2:N9" si="5">M2-L2</f>
         <v>0</v>
       </c>
       <c r="O2" t="s">
         <v>9</v>
       </c>
       <c r="P2">
-        <v>143</v>
+        <v>3364</v>
       </c>
       <c r="Q2">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2" s="4">
+        <v>7</v>
+      </c>
+      <c r="S2" s="3">
         <v>50645.33</v>
       </c>
       <c r="T2">
-        <f>D2/S2</f>
+        <f t="shared" ref="T2:T33" si="6">D2/S2</f>
         <v>99.319186981307055</v>
       </c>
       <c r="U2">
@@ -1447,11 +1439,11 @@
       <c r="Y2">
         <v>43</v>
       </c>
-      <c r="Z2" s="5">
+      <c r="Z2" s="4">
         <v>1240000</v>
       </c>
-      <c r="AA2" s="6">
-        <f>Z2/D2</f>
+      <c r="AA2" s="5">
+        <f t="shared" ref="AA2:AA33" si="7">Z2/D2</f>
         <v>0.2465182772428044</v>
       </c>
     </row>
@@ -1460,7 +1452,7 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C3">
         <v>721523</v>
@@ -1472,15 +1464,15 @@
         <v>731158</v>
       </c>
       <c r="F3">
-        <f>D3-C3</f>
+        <f t="shared" si="0"/>
         <v>14558</v>
       </c>
       <c r="G3">
-        <f>F3/C3*100</f>
+        <f t="shared" si="1"/>
         <v>2.0176764981850894</v>
       </c>
       <c r="H3" s="2">
-        <f>(D3-E3)/E3</f>
+        <f t="shared" si="2"/>
         <v>6.7331548037496683E-3</v>
       </c>
       <c r="I3">
@@ -1490,37 +1482,37 @@
         <v>1</v>
       </c>
       <c r="K3">
-        <f>J3-I3</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L3">
         <v>3</v>
       </c>
       <c r="M3">
-        <f>J3+2</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="N3">
-        <f>M3-L3</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="O3" t="s">
         <v>9</v>
       </c>
       <c r="P3">
-        <v>1106</v>
+        <v>141</v>
       </c>
       <c r="Q3">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="R3">
-        <v>4</v>
-      </c>
-      <c r="S3" s="4">
+        <v>0</v>
+      </c>
+      <c r="S3" s="3">
         <v>570640.94999999995</v>
       </c>
       <c r="T3">
-        <f>D3/S3</f>
+        <f t="shared" si="6"/>
         <v>1.289919694687176</v>
       </c>
       <c r="U3">
@@ -1538,11 +1530,11 @@
       <c r="Y3">
         <v>32</v>
       </c>
-      <c r="Z3" s="5">
+      <c r="Z3" s="4">
         <v>600000</v>
       </c>
-      <c r="AA3" s="6">
-        <f>Z3/D3</f>
+      <c r="AA3" s="5">
+        <f t="shared" si="7"/>
         <v>0.81512768295880478</v>
       </c>
     </row>
@@ -1563,15 +1555,15 @@
         <v>7421401</v>
       </c>
       <c r="F4">
-        <f>D4-C4</f>
+        <f t="shared" si="0"/>
         <v>746223</v>
       </c>
       <c r="G4">
-        <f>F4/C4*100</f>
+        <f t="shared" si="1"/>
         <v>11.636642911722053</v>
       </c>
       <c r="H4" s="2">
-        <f>(D4-E4)/E4</f>
+        <f t="shared" si="2"/>
         <v>-3.5367715610570026E-2</v>
       </c>
       <c r="I4">
@@ -1581,18 +1573,18 @@
         <v>9</v>
       </c>
       <c r="K4">
-        <f>J4-I4</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L4">
         <v>11</v>
       </c>
       <c r="M4">
-        <f>J4+2</f>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="N4">
-        <f>M4-L4</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="O4" t="s">
@@ -1607,11 +1599,11 @@
       <c r="R4">
         <v>5</v>
       </c>
-      <c r="S4" s="4">
+      <c r="S4" s="3">
         <v>113594.08</v>
       </c>
       <c r="T4">
-        <f>D4/S4</f>
+        <f t="shared" si="6"/>
         <v>63.021972623925471</v>
       </c>
       <c r="U4">
@@ -1629,11 +1621,11 @@
       <c r="Y4">
         <v>25</v>
       </c>
-      <c r="Z4" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="6">
-        <f>Z4/D4</f>
+      <c r="Z4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -1654,15 +1646,15 @@
         <v>3030522</v>
       </c>
       <c r="F5">
-        <f>D5-C5</f>
+        <f t="shared" si="0"/>
         <v>87527</v>
       </c>
       <c r="G5">
-        <f>F5/C5*100</f>
+        <f t="shared" si="1"/>
         <v>2.9911192869730976</v>
       </c>
       <c r="H5" s="2">
-        <f>(D5-E5)/E5</f>
+        <f t="shared" si="2"/>
         <v>-5.5323802302045654E-3</v>
       </c>
       <c r="I5">
@@ -1672,18 +1664,18 @@
         <v>4</v>
       </c>
       <c r="K5">
-        <f>J5-I5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L5">
         <v>6</v>
       </c>
       <c r="M5">
-        <f>J5+2</f>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="N5">
-        <f>M5-L5</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="O5" t="s">
@@ -1698,11 +1690,11 @@
       <c r="R5">
         <v>2</v>
       </c>
-      <c r="S5" s="4">
+      <c r="S5" s="3">
         <v>52035.48</v>
       </c>
       <c r="T5">
-        <f>D5/S5</f>
+        <f t="shared" si="6"/>
         <v>57.917328714946031</v>
       </c>
       <c r="U5">
@@ -1720,11 +1712,11 @@
       <c r="Y5">
         <v>46</v>
       </c>
-      <c r="Z5" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="6">
-        <f>Z5/D5</f>
+      <c r="Z5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -1745,15 +1737,15 @@
         <v>39368078</v>
       </c>
       <c r="F6">
-        <f>D6-C6</f>
+        <f t="shared" si="0"/>
         <v>2234768</v>
       </c>
       <c r="G6">
-        <f>F6/C6*100</f>
+        <f t="shared" si="1"/>
         <v>5.9845981958807819</v>
       </c>
       <c r="H6" s="2">
-        <f>(D6-E6)/E6</f>
+        <f t="shared" si="2"/>
         <v>5.3007159760250422E-3</v>
       </c>
       <c r="I6">
@@ -1763,18 +1755,18 @@
         <v>52</v>
       </c>
       <c r="K6">
-        <f>J6-I6</f>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
       <c r="L6">
         <v>55</v>
       </c>
       <c r="M6">
-        <f>J6+2</f>
+        <f t="shared" si="4"/>
         <v>54</v>
       </c>
       <c r="N6">
-        <f>M6-L6</f>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
       <c r="O6" t="s">
@@ -1789,11 +1781,11 @@
       <c r="R6">
         <v>0</v>
       </c>
-      <c r="S6" s="4">
+      <c r="S6" s="3">
         <v>155779.22</v>
       </c>
       <c r="T6">
-        <f>D6/S6</f>
+        <f t="shared" si="6"/>
         <v>254.05671565180515</v>
       </c>
       <c r="U6">
@@ -1811,11 +1803,11 @@
       <c r="Y6">
         <v>6</v>
       </c>
-      <c r="Z6" s="5">
+      <c r="Z6" s="4">
         <v>187000000</v>
       </c>
-      <c r="AA6" s="6">
-        <f>Z6/D6</f>
+      <c r="AA6" s="5">
+        <f t="shared" si="7"/>
         <v>4.7249955320998129</v>
       </c>
     </row>
@@ -1836,15 +1828,15 @@
         <v>5807719</v>
       </c>
       <c r="F7">
-        <f>D7-C7</f>
+        <f t="shared" si="0"/>
         <v>737241</v>
       </c>
       <c r="G7">
-        <f>F7/C7*100</f>
+        <f t="shared" si="1"/>
         <v>14.613503061489455</v>
       </c>
       <c r="H7" s="2">
-        <f>(D7-E7)/E7</f>
+        <f t="shared" si="2"/>
         <v>-4.3989731596862725E-3</v>
       </c>
       <c r="I7">
@@ -1854,18 +1846,18 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <f>J7-I7</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L7">
         <v>9</v>
       </c>
       <c r="M7">
-        <f>J7+2</f>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N7">
-        <f>M7-L7</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="O7" t="s">
@@ -1880,11 +1872,11 @@
       <c r="R7">
         <v>11</v>
       </c>
-      <c r="S7" s="4">
+      <c r="S7" s="3">
         <v>103641.89</v>
       </c>
       <c r="T7">
-        <f>D7/S7</f>
+        <f t="shared" si="6"/>
         <v>55.789903098061991</v>
       </c>
       <c r="U7">
@@ -1902,11 +1894,11 @@
       <c r="Y7">
         <v>15</v>
       </c>
-      <c r="Z7" s="5">
+      <c r="Z7" s="4">
         <v>6000000</v>
       </c>
-      <c r="AA7" s="6">
-        <f>Z7/D7</f>
+      <c r="AA7" s="5">
+        <f t="shared" si="7"/>
         <v>1.0376725281905361</v>
       </c>
     </row>
@@ -1927,15 +1919,15 @@
         <v>3557006</v>
       </c>
       <c r="F8">
-        <f>D8-C8</f>
+        <f t="shared" si="0"/>
         <v>26670</v>
       </c>
       <c r="G8">
-        <f>F8/C8*100</f>
+        <f t="shared" si="1"/>
         <v>0.74463344601951964</v>
       </c>
       <c r="H8" s="2">
-        <f>(D8-E8)/E8</f>
+        <f t="shared" si="2"/>
         <v>1.4419992544291464E-2</v>
       </c>
       <c r="I8">
@@ -1945,18 +1937,18 @@
         <v>5</v>
       </c>
       <c r="K8">
-        <f>J8-I8</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L8">
         <v>7</v>
       </c>
       <c r="M8">
-        <f>J8+2</f>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="N8">
-        <f>M8-L8</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="O8" t="s">
@@ -1971,11 +1963,11 @@
       <c r="R8">
         <v>16</v>
       </c>
-      <c r="S8" s="4">
+      <c r="S8" s="3">
         <v>4842.3599999999997</v>
       </c>
       <c r="T8">
-        <f>D8/S8</f>
+        <f t="shared" si="6"/>
         <v>745.15277674522349</v>
       </c>
       <c r="U8">
@@ -1993,11 +1985,11 @@
       <c r="Y8">
         <v>9</v>
       </c>
-      <c r="Z8" s="5">
+      <c r="Z8" s="4">
         <v>500000</v>
       </c>
-      <c r="AA8" s="6">
-        <f>Z8/D8</f>
+      <c r="AA8" s="5">
+        <f t="shared" si="7"/>
         <v>0.13856948622314455</v>
       </c>
     </row>
@@ -2018,15 +2010,15 @@
         <v>986809</v>
       </c>
       <c r="F9">
-        <f>D9-C9</f>
+        <f t="shared" si="0"/>
         <v>89960</v>
       </c>
       <c r="G9">
-        <f>F9/C9*100</f>
+        <f t="shared" si="1"/>
         <v>9.9858249239352332</v>
       </c>
       <c r="H9" s="2">
-        <f>(D9-E9)/E9</f>
+        <f t="shared" si="2"/>
         <v>4.0818435989132653E-3</v>
       </c>
       <c r="I9">
@@ -2036,18 +2028,18 @@
         <v>1</v>
       </c>
       <c r="K9">
-        <f>J9-I9</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L9">
         <v>3</v>
       </c>
       <c r="M9">
-        <f>J9+2</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="N9">
-        <f>M9-L9</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="O9" t="s">
@@ -2062,11 +2054,11 @@
       <c r="R9">
         <v>1</v>
       </c>
-      <c r="S9" s="4">
+      <c r="S9" s="3">
         <v>1948.54</v>
       </c>
       <c r="T9">
-        <f>D9/S9</f>
+        <f t="shared" si="6"/>
         <v>508.50226323298472</v>
       </c>
       <c r="U9">
@@ -2084,11 +2076,11 @@
       <c r="Y9">
         <v>11</v>
       </c>
-      <c r="Z9" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA9" s="6">
-        <f>Z9/D9</f>
+      <c r="Z9" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2110,15 +2102,15 @@
         <v>712816</v>
       </c>
       <c r="F10">
-        <f>D10-C10</f>
+        <f t="shared" si="0"/>
         <v>89810</v>
       </c>
       <c r="G10">
-        <f>F10/C10*100</f>
+        <f t="shared" si="1"/>
         <v>14.925472351896138</v>
       </c>
       <c r="H10" s="2">
-        <f>(D10-E10)/E10</f>
+        <f t="shared" si="2"/>
         <v>-2.9857635069919865E-2</v>
       </c>
       <c r="I10">
@@ -2128,7 +2120,7 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <f>J10-I10</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L10">
@@ -2156,7 +2148,7 @@
         <v>61.05</v>
       </c>
       <c r="T10">
-        <f>D10/S10</f>
+        <f t="shared" si="6"/>
         <v>11327.321867321867</v>
       </c>
       <c r="U10">
@@ -2174,11 +2166,11 @@
       <c r="Y10">
         <v>1</v>
       </c>
-      <c r="Z10" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="6">
-        <f>Z10/D10</f>
+      <c r="Z10" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2199,15 +2191,15 @@
         <v>21733312</v>
       </c>
       <c r="F11">
-        <f>D11-C11</f>
+        <f t="shared" si="0"/>
         <v>2669754</v>
       </c>
       <c r="G11">
-        <f>F11/C11*100</f>
+        <f t="shared" si="1"/>
         <v>14.12510483036858</v>
       </c>
       <c r="H11" s="2">
-        <f>(D11-E11)/E11</f>
+        <f t="shared" si="2"/>
         <v>-7.4901147142230323E-3</v>
       </c>
       <c r="I11">
@@ -2217,18 +2209,18 @@
         <v>28</v>
       </c>
       <c r="K11">
-        <f>J11-I11</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L11">
         <v>29</v>
       </c>
       <c r="M11">
-        <f>J11+2</f>
+        <f t="shared" ref="M11:M52" si="8">J11+2</f>
         <v>30</v>
       </c>
       <c r="N11">
-        <f>M11-L11</f>
+        <f t="shared" ref="N11:N52" si="9">M11-L11</f>
         <v>1</v>
       </c>
       <c r="O11" t="s">
@@ -2243,11 +2235,11 @@
       <c r="R11">
         <v>16</v>
       </c>
-      <c r="S11" s="4">
+      <c r="S11" s="3">
         <v>53624.76</v>
       </c>
       <c r="T11">
-        <f>D11/S11</f>
+        <f t="shared" si="6"/>
         <v>402.24939002058005</v>
       </c>
       <c r="U11">
@@ -2265,11 +2257,11 @@
       <c r="Y11">
         <v>28</v>
       </c>
-      <c r="Z11" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="6">
-        <f>Z11/D11</f>
+      <c r="Z11" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2290,15 +2282,15 @@
         <v>10710017</v>
       </c>
       <c r="F12">
-        <f>D12-C12</f>
+        <f t="shared" si="0"/>
         <v>997708</v>
       </c>
       <c r="G12">
-        <f>F12/C12*100</f>
+        <f t="shared" si="1"/>
         <v>10.256501986211145</v>
       </c>
       <c r="H12" s="2">
-        <f>(D12-E12)/E12</f>
+        <f t="shared" si="2"/>
         <v>1.4245542280651841E-3</v>
       </c>
       <c r="I12">
@@ -2308,18 +2300,18 @@
         <v>14</v>
       </c>
       <c r="K12">
-        <f>J12-I12</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L12">
         <v>16</v>
       </c>
       <c r="M12">
-        <f>J12+2</f>
+        <f t="shared" si="8"/>
         <v>16</v>
       </c>
       <c r="N12">
-        <f>M12-L12</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O12" t="s">
@@ -2334,11 +2326,11 @@
       <c r="R12">
         <v>24</v>
       </c>
-      <c r="S12" s="4">
+      <c r="S12" s="3">
         <v>57513.49</v>
       </c>
       <c r="T12">
-        <f>D12/S12</f>
+        <f t="shared" si="6"/>
         <v>186.48275387217851</v>
       </c>
       <c r="U12">
@@ -2356,11 +2348,11 @@
       <c r="Y12">
         <v>26</v>
       </c>
-      <c r="Z12" s="5">
+      <c r="Z12" s="4">
         <v>3750886</v>
       </c>
-      <c r="AA12" s="6">
-        <f>Z12/D12</f>
+      <c r="AA12" s="5">
+        <f t="shared" si="7"/>
         <v>0.34972402569855093</v>
       </c>
     </row>
@@ -2381,15 +2373,15 @@
         <v>1407006</v>
       </c>
       <c r="F13">
-        <f>D13-C13</f>
+        <f t="shared" si="0"/>
         <v>93275</v>
       </c>
       <c r="G13">
-        <f>F13/C13*100</f>
+        <f t="shared" si="1"/>
         <v>6.8240246637919553</v>
       </c>
       <c r="H13" s="2">
-        <f>(D13-E13)/E13</f>
+        <f t="shared" si="2"/>
         <v>3.7761743731014652E-2</v>
       </c>
       <c r="I13">
@@ -2399,18 +2391,18 @@
         <v>2</v>
       </c>
       <c r="K13">
-        <f>J13-I13</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L13">
         <v>4</v>
       </c>
       <c r="M13">
-        <f>J13+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N13">
-        <f>M13-L13</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O13" t="s">
@@ -2425,11 +2417,11 @@
       <c r="R13">
         <v>0</v>
       </c>
-      <c r="S13" s="4">
+      <c r="S13" s="3">
         <v>6422.63</v>
       </c>
       <c r="T13">
-        <f>D13/S13</f>
+        <f t="shared" si="6"/>
         <v>227.34253724720247</v>
       </c>
       <c r="U13">
@@ -2447,11 +2439,11 @@
       <c r="Y13">
         <v>5</v>
       </c>
-      <c r="Z13" s="5">
+      <c r="Z13" s="4">
         <v>750000</v>
       </c>
-      <c r="AA13" s="6">
-        <f>Z13/D13</f>
+      <c r="AA13" s="5">
+        <f t="shared" si="7"/>
         <v>0.51365043143211908</v>
       </c>
     </row>
@@ -2472,15 +2464,15 @@
         <v>1826913</v>
       </c>
       <c r="F14">
-        <f>D14-C14</f>
+        <f t="shared" si="0"/>
         <v>267878</v>
       </c>
       <c r="G14">
-        <f>F14/C14*100</f>
+        <f t="shared" si="1"/>
         <v>17.024351461297403</v>
       </c>
       <c r="H14" s="2">
-        <f>(D14-E14)/E14</f>
+        <f t="shared" si="2"/>
         <v>7.9171805116061908E-3</v>
       </c>
       <c r="I14">
@@ -2490,18 +2482,18 @@
         <v>2</v>
       </c>
       <c r="K14">
-        <f>J14-I14</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L14">
         <v>4</v>
       </c>
       <c r="M14">
-        <f>J14+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N14">
-        <f>M14-L14</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O14" t="s">
@@ -2516,11 +2508,11 @@
       <c r="R14">
         <v>0</v>
       </c>
-      <c r="S14" s="4">
+      <c r="S14" s="3">
         <v>82643.12</v>
       </c>
       <c r="T14">
-        <f>D14/S14</f>
+        <f t="shared" si="6"/>
         <v>22.281068284934065</v>
       </c>
       <c r="U14">
@@ -2538,11 +2530,11 @@
       <c r="Y14">
         <v>47</v>
       </c>
-      <c r="Z14" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="6">
-        <f>Z14/D14</f>
+      <c r="Z14" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2563,15 +2555,15 @@
         <v>12587530</v>
       </c>
       <c r="F15">
-        <f>D15-C15</f>
+        <f t="shared" si="0"/>
         <v>-41641</v>
       </c>
       <c r="G15">
-        <f>F15/C15*100</f>
+        <f t="shared" si="1"/>
         <v>-0.32369224167818428</v>
       </c>
       <c r="H15" s="2">
-        <f>(D15-E15)/E15</f>
+        <f t="shared" si="2"/>
         <v>1.8685874035652746E-2</v>
       </c>
       <c r="I15">
@@ -2581,18 +2573,18 @@
         <v>17</v>
       </c>
       <c r="K15">
-        <f>J15-I15</f>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
       <c r="L15">
         <v>20</v>
       </c>
       <c r="M15">
-        <f>J15+2</f>
+        <f t="shared" si="8"/>
         <v>19</v>
       </c>
       <c r="N15">
-        <f>M15-L15</f>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="O15" t="s">
@@ -2607,11 +2599,11 @@
       <c r="R15">
         <v>42</v>
       </c>
-      <c r="S15" s="4">
+      <c r="S15" s="3">
         <v>55518.93</v>
       </c>
       <c r="T15">
-        <f>D15/S15</f>
+        <f t="shared" si="6"/>
         <v>230.96156572181778</v>
       </c>
       <c r="U15">
@@ -2629,11 +2621,11 @@
       <c r="Y15">
         <v>12</v>
       </c>
-      <c r="Z15" s="5">
+      <c r="Z15" s="4">
         <v>30500000</v>
       </c>
-      <c r="AA15" s="6">
-        <f>Z15/D15</f>
+      <c r="AA15" s="5">
+        <f t="shared" si="7"/>
         <v>2.3785869774000701</v>
       </c>
     </row>
@@ -2654,15 +2646,15 @@
         <v>6754953</v>
       </c>
       <c r="F16">
-        <f>D16-C16</f>
+        <f t="shared" si="0"/>
         <v>288698</v>
       </c>
       <c r="G16">
-        <f>F16/C16*100</f>
+        <f t="shared" si="1"/>
         <v>4.4404269606997193</v>
       </c>
       <c r="H16" s="2">
-        <f>(D16-E16)/E16</f>
+        <f t="shared" si="2"/>
         <v>5.2297921243863576E-3</v>
       </c>
       <c r="I16">
@@ -2672,18 +2664,18 @@
         <v>9</v>
       </c>
       <c r="K16">
-        <f>J16-I16</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L16">
         <v>11</v>
       </c>
       <c r="M16">
-        <f>J16+2</f>
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
       <c r="N16">
-        <f>M16-L16</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O16" t="s">
@@ -2698,11 +2690,11 @@
       <c r="R16">
         <v>16</v>
       </c>
-      <c r="S16" s="4">
+      <c r="S16" s="3">
         <v>35826.11</v>
       </c>
       <c r="T16">
-        <f>D16/S16</f>
+        <f t="shared" si="6"/>
         <v>189.53439265384938</v>
       </c>
       <c r="U16">
@@ -2720,11 +2712,11 @@
       <c r="Y16">
         <v>36</v>
       </c>
-      <c r="Z16" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="6">
-        <f>Z16/D16</f>
+      <c r="Z16" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2745,15 +2737,15 @@
         <v>3163561</v>
       </c>
       <c r="F17">
-        <f>D17-C17</f>
+        <f t="shared" si="0"/>
         <v>138619</v>
       </c>
       <c r="G17">
-        <f>F17/C17*100</f>
+        <f t="shared" si="1"/>
         <v>4.5392491355814926</v>
       </c>
       <c r="H17" s="2">
-        <f>(D17-E17)/E17</f>
+        <f t="shared" si="2"/>
         <v>9.1178896186923531E-3</v>
       </c>
       <c r="I17">
@@ -2763,18 +2755,18 @@
         <v>4</v>
       </c>
       <c r="K17">
-        <f>J17-I17</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L17">
         <v>6</v>
       </c>
       <c r="M17">
-        <f>J17+2</f>
+        <f t="shared" si="8"/>
         <v>6</v>
       </c>
       <c r="N17">
-        <f>M17-L17</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O17" t="s">
@@ -2789,11 +2781,11 @@
       <c r="R17">
         <v>2</v>
       </c>
-      <c r="S17" s="4">
+      <c r="S17" s="3">
         <v>55857.13</v>
       </c>
       <c r="T17">
-        <f>D17/S17</f>
+        <f t="shared" si="6"/>
         <v>57.153061748786591</v>
       </c>
       <c r="U17">
@@ -2811,11 +2803,11 @@
       <c r="Y17">
         <v>31</v>
       </c>
-      <c r="Z17" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="6">
-        <f>Z17/D17</f>
+      <c r="Z17" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2836,15 +2828,15 @@
         <v>2913805</v>
       </c>
       <c r="F18">
-        <f>D18-C18</f>
+        <f t="shared" si="0"/>
         <v>77052</v>
       </c>
       <c r="G18">
-        <f>F18/C18*100</f>
+        <f t="shared" si="1"/>
         <v>2.6905388026383008</v>
       </c>
       <c r="H18" s="2">
-        <f>(D18-E18)/E18</f>
+        <f t="shared" si="2"/>
         <v>9.2868259886986267E-3</v>
       </c>
       <c r="I18">
@@ -2854,18 +2846,18 @@
         <v>4</v>
       </c>
       <c r="K18">
-        <f>J18-I18</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L18">
         <v>6</v>
       </c>
       <c r="M18">
-        <f>J18+2</f>
+        <f t="shared" si="8"/>
         <v>6</v>
       </c>
       <c r="N18">
-        <f>M18-L18</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O18" t="s">
@@ -2880,11 +2872,11 @@
       <c r="R18">
         <v>1</v>
       </c>
-      <c r="S18" s="4">
+      <c r="S18" s="3">
         <v>81758.720000000001</v>
       </c>
       <c r="T18">
-        <f>D18/S18</f>
+        <f t="shared" si="6"/>
         <v>35.97004698703698</v>
       </c>
       <c r="U18">
@@ -2902,11 +2894,11 @@
       <c r="Y18">
         <v>34</v>
       </c>
-      <c r="Z18" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="6">
-        <f>Z18/D18</f>
+      <c r="Z18" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2927,15 +2919,15 @@
         <v>4477251</v>
       </c>
       <c r="F19">
-        <f>D19-C19</f>
+        <f t="shared" si="0"/>
         <v>158736</v>
       </c>
       <c r="G19">
-        <f>F19/C19*100</f>
+        <f t="shared" si="1"/>
         <v>3.6485951612258156</v>
       </c>
       <c r="H19" s="2">
-        <f>(D19-E19)/E19</f>
+        <f t="shared" si="2"/>
         <v>7.1675677776385557E-3</v>
       </c>
       <c r="I19">
@@ -2945,18 +2937,18 @@
         <v>6</v>
       </c>
       <c r="K19">
-        <f>J19-I19</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L19">
         <v>8</v>
       </c>
       <c r="M19">
-        <f>J19+2</f>
+        <f t="shared" si="8"/>
         <v>8</v>
       </c>
       <c r="N19">
-        <f>M19-L19</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O19" t="s">
@@ -2971,11 +2963,11 @@
       <c r="R19">
         <v>2</v>
       </c>
-      <c r="S19" s="4">
+      <c r="S19" s="3">
         <v>39486.339999999997</v>
       </c>
       <c r="T19">
-        <f>D19/S19</f>
+        <f t="shared" si="6"/>
         <v>114.2000499413215</v>
       </c>
       <c r="U19">
@@ -2993,11 +2985,11 @@
       <c r="Y19">
         <v>44</v>
       </c>
-      <c r="Z19" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="6">
-        <f>Z19/D19</f>
+      <c r="Z19" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3018,15 +3010,15 @@
         <v>4645318</v>
       </c>
       <c r="F20">
-        <f>D20-C20</f>
+        <f t="shared" si="0"/>
         <v>107506</v>
       </c>
       <c r="G20">
-        <f>F20/C20*100</f>
+        <f t="shared" si="1"/>
         <v>2.3607135940089092</v>
       </c>
       <c r="H20" s="2">
-        <f>(D20-E20)/E20</f>
+        <f t="shared" si="2"/>
         <v>3.4766188235121902E-3</v>
       </c>
       <c r="I20">
@@ -3036,18 +3028,18 @@
         <v>6</v>
       </c>
       <c r="K20">
-        <f>J20-I20</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L20">
         <v>8</v>
       </c>
       <c r="M20">
-        <f>J20+2</f>
+        <f t="shared" si="8"/>
         <v>8</v>
       </c>
       <c r="N20">
-        <f>M20-L20</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O20" t="s">
@@ -3062,11 +3054,11 @@
       <c r="R20">
         <v>34</v>
       </c>
-      <c r="S20" s="4">
+      <c r="S20" s="3">
         <v>43203.9</v>
       </c>
       <c r="T20">
-        <f>D20/S20</f>
+        <f t="shared" si="6"/>
         <v>107.89461136610352</v>
       </c>
       <c r="U20">
@@ -3084,11 +3076,11 @@
       <c r="Y20">
         <v>39</v>
       </c>
-      <c r="Z20" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="6">
-        <f>Z20/D20</f>
+      <c r="Z20" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3109,15 +3101,15 @@
         <v>1350141</v>
       </c>
       <c r="F21">
-        <f>D21-C21</f>
+        <f t="shared" si="0"/>
         <v>30508</v>
       </c>
       <c r="G21">
-        <f>F21/C21*100</f>
+        <f t="shared" si="1"/>
         <v>2.2885451220262341</v>
       </c>
       <c r="H21" s="2">
-        <f>(D21-E21)/E21</f>
+        <f t="shared" si="2"/>
         <v>9.9552565250592348E-3</v>
       </c>
       <c r="I21">
@@ -3127,18 +3119,18 @@
         <v>2</v>
       </c>
       <c r="K21">
-        <f>J21-I21</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L21">
         <v>4</v>
       </c>
       <c r="M21">
-        <f>J21+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N21">
-        <f>M21-L21</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O21" t="s">
@@ -3153,11 +3145,11 @@
       <c r="R21">
         <v>2</v>
       </c>
-      <c r="S21" s="4">
+      <c r="S21" s="3">
         <v>30842.92</v>
       </c>
       <c r="T21">
-        <f>D21/S21</f>
+        <f t="shared" si="6"/>
         <v>44.210535189275205</v>
       </c>
       <c r="U21">
@@ -3175,11 +3167,11 @@
       <c r="Y21">
         <v>18</v>
       </c>
-      <c r="Z21" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="6">
-        <f>Z21/D21</f>
+      <c r="Z21" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3200,15 +3192,15 @@
         <v>6055802</v>
       </c>
       <c r="F22">
-        <f>D22-C22</f>
+        <f t="shared" si="0"/>
         <v>395349</v>
       </c>
       <c r="G22">
-        <f>F22/C22*100</f>
+        <f t="shared" si="1"/>
         <v>6.8282184462020172</v>
       </c>
       <c r="H22" s="2">
-        <f>(D22-E22)/E22</f>
+        <f t="shared" si="2"/>
         <v>2.1380487671162299E-2</v>
       </c>
       <c r="I22">
@@ -3218,18 +3210,18 @@
         <v>8</v>
       </c>
       <c r="K22">
-        <f>J22-I22</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L22">
         <v>10</v>
       </c>
       <c r="M22">
-        <f>J22+2</f>
+        <f t="shared" si="8"/>
         <v>10</v>
       </c>
       <c r="N22">
-        <f>M22-L22</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O22" t="s">
@@ -3244,11 +3236,11 @@
       <c r="R22">
         <v>13</v>
       </c>
-      <c r="S22" s="4">
+      <c r="S22" s="3">
         <v>9707.24</v>
       </c>
       <c r="T22">
-        <f>D22/S22</f>
+        <f t="shared" si="6"/>
         <v>637.18193842946096</v>
       </c>
       <c r="U22">
@@ -3266,11 +3258,11 @@
       <c r="Y22">
         <v>4</v>
       </c>
-      <c r="Z22" s="5">
+      <c r="Z22" s="4">
         <v>5000000</v>
       </c>
-      <c r="AA22" s="6">
-        <f>Z22/D22</f>
+      <c r="AA22" s="5">
+        <f t="shared" si="7"/>
         <v>0.80837110312584171</v>
       </c>
     </row>
@@ -3291,15 +3283,15 @@
         <v>6893574</v>
       </c>
       <c r="F23">
-        <f>D23-C23</f>
+        <f t="shared" si="0"/>
         <v>473825</v>
       </c>
       <c r="G23">
-        <f>F23/C23*100</f>
+        <f t="shared" si="1"/>
         <v>7.223334071178253</v>
       </c>
       <c r="H23" s="2">
-        <f>(D23-E23)/E23</f>
+        <f t="shared" si="2"/>
         <v>2.0293537140531167E-2</v>
       </c>
       <c r="I23">
@@ -3309,18 +3301,18 @@
         <v>9</v>
       </c>
       <c r="K23">
-        <f>J23-I23</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L23">
         <v>11</v>
       </c>
       <c r="M23">
-        <f>J23+2</f>
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
       <c r="N23">
-        <f>M23-L23</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O23" t="s">
@@ -3335,11 +3327,11 @@
       <c r="R23">
         <v>33</v>
       </c>
-      <c r="S23" s="4">
+      <c r="S23" s="3">
         <v>7800.06</v>
       </c>
       <c r="T23">
-        <f>D23/S23</f>
+        <f t="shared" si="6"/>
         <v>901.71985856519052</v>
       </c>
       <c r="U23">
@@ -3357,11 +3349,11 @@
       <c r="Y23">
         <v>3</v>
       </c>
-      <c r="Z23" s="5">
+      <c r="Z23" s="4">
         <v>6650000</v>
       </c>
-      <c r="AA23" s="6">
-        <f>Z23/D23</f>
+      <c r="AA23" s="5">
+        <f t="shared" si="7"/>
         <v>0.94547939288564431</v>
       </c>
     </row>
@@ -3382,15 +3374,15 @@
         <v>9966555</v>
       </c>
       <c r="F24">
-        <f>D24-C24</f>
+        <f t="shared" si="0"/>
         <v>172816</v>
       </c>
       <c r="G24">
-        <f>F24/C24*100</f>
+        <f t="shared" si="1"/>
         <v>1.743568613262849</v>
       </c>
       <c r="H24" s="2">
-        <f>(D24-E24)/E24</f>
+        <f t="shared" si="2"/>
         <v>1.1828259614279959E-2</v>
       </c>
       <c r="I24">
@@ -3400,18 +3392,18 @@
         <v>13</v>
       </c>
       <c r="K24">
-        <f>J24-I24</f>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
       <c r="L24">
         <v>16</v>
       </c>
       <c r="M24">
-        <f>J24+2</f>
+        <f t="shared" si="8"/>
         <v>15</v>
       </c>
       <c r="N24">
-        <f>M24-L24</f>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="O24" t="s">
@@ -3426,11 +3418,11 @@
       <c r="R24">
         <v>78</v>
       </c>
-      <c r="S24" s="4">
+      <c r="S24" s="3">
         <v>56538.9</v>
       </c>
       <c r="T24">
-        <f>D24/S24</f>
+        <f t="shared" si="6"/>
         <v>178.36289704964193</v>
       </c>
       <c r="U24">
@@ -3448,11 +3440,11 @@
       <c r="Y24">
         <v>21</v>
       </c>
-      <c r="Z24" s="5">
+      <c r="Z24" s="4">
         <v>16000000</v>
       </c>
-      <c r="AA24" s="6">
-        <f>Z24/D24</f>
+      <c r="AA24" s="5">
+        <f t="shared" si="7"/>
         <v>1.5866024119133215</v>
       </c>
     </row>
@@ -3473,15 +3465,15 @@
         <v>5657342</v>
       </c>
       <c r="F25">
-        <f>D25-C25</f>
+        <f t="shared" si="0"/>
         <v>394873</v>
       </c>
       <c r="G25">
-        <f>F25/C25*100</f>
+        <f t="shared" si="1"/>
         <v>7.4295764776582871</v>
       </c>
       <c r="H25" s="2">
-        <f>(D25-E25)/E25</f>
+        <f t="shared" si="2"/>
         <v>9.2640678254911936E-3</v>
       </c>
       <c r="I25">
@@ -3491,18 +3483,18 @@
         <v>8</v>
       </c>
       <c r="K25">
-        <f>J25-I25</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L25">
         <v>10</v>
       </c>
       <c r="M25">
-        <f>J25+2</f>
+        <f t="shared" si="8"/>
         <v>10</v>
       </c>
       <c r="N25">
-        <f>M25-L25</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O25" t="s">
@@ -3517,11 +3509,11 @@
       <c r="R25">
         <v>1</v>
       </c>
-      <c r="S25" s="4">
+      <c r="S25" s="3">
         <v>79626.740000000005</v>
       </c>
       <c r="T25">
-        <f>D25/S25</f>
+        <f t="shared" si="6"/>
         <v>71.706464436444335</v>
       </c>
       <c r="U25">
@@ -3539,11 +3531,11 @@
       <c r="Y25">
         <v>20</v>
       </c>
-      <c r="Z25" s="5">
+      <c r="Z25" s="4">
         <v>2170000</v>
       </c>
-      <c r="AA25" s="6">
-        <f>Z25/D25</f>
+      <c r="AA25" s="5">
+        <f t="shared" si="7"/>
         <v>0.38005153288619192</v>
       </c>
     </row>
@@ -3564,15 +3556,15 @@
         <v>2966786</v>
       </c>
       <c r="F26">
-        <f>D26-C26</f>
+        <f t="shared" si="0"/>
         <v>-14326</v>
       </c>
       <c r="G26">
-        <f>F26/C26*100</f>
+        <f t="shared" si="1"/>
         <v>-0.48102234876974315</v>
       </c>
       <c r="H26" s="2">
-        <f>(D26-E26)/E26</f>
+        <f t="shared" si="2"/>
         <v>-9.6805094806298806E-4</v>
       </c>
       <c r="I26">
@@ -3582,18 +3574,18 @@
         <v>4</v>
       </c>
       <c r="K26">
-        <f>J26-I26</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L26">
         <v>6</v>
       </c>
       <c r="M26">
-        <f>J26+2</f>
+        <f t="shared" si="8"/>
         <v>6</v>
       </c>
       <c r="N26">
-        <f>M26-L26</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O26" t="s">
@@ -3608,11 +3600,11 @@
       <c r="R26">
         <v>4</v>
       </c>
-      <c r="S26" s="4">
+      <c r="S26" s="3">
         <v>46923.27</v>
       </c>
       <c r="T26">
-        <f>D26/S26</f>
+        <f t="shared" si="6"/>
         <v>63.165120418930741</v>
       </c>
       <c r="U26">
@@ -3630,11 +3622,11 @@
       <c r="Y26">
         <v>37</v>
       </c>
-      <c r="Z26" s="5">
+      <c r="Z26" s="4">
         <v>400000</v>
       </c>
-      <c r="AA26" s="6">
-        <f>Z26/D26</f>
+      <c r="AA26" s="5">
+        <f t="shared" si="7"/>
         <v>0.13495668227890553</v>
       </c>
     </row>
@@ -3655,15 +3647,15 @@
         <v>6151548</v>
       </c>
       <c r="F27">
-        <f>D27-C27</f>
+        <f t="shared" si="0"/>
         <v>148803</v>
       </c>
       <c r="G27">
-        <f>F27/C27*100</f>
+        <f t="shared" si="1"/>
         <v>2.4753147229350252</v>
       </c>
       <c r="H27" s="2">
-        <f>(D27-E27)/E27</f>
+        <f t="shared" si="2"/>
         <v>1.4196426655534509E-3</v>
       </c>
       <c r="I27">
@@ -3673,18 +3665,18 @@
         <v>8</v>
       </c>
       <c r="K27">
-        <f>J27-I27</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L27">
         <v>10</v>
       </c>
       <c r="M27">
-        <f>J27+2</f>
+        <f t="shared" si="8"/>
         <v>10</v>
       </c>
       <c r="N27">
-        <f>M27-L27</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O27" t="s">
@@ -3699,11 +3691,11 @@
       <c r="R27">
         <v>4</v>
       </c>
-      <c r="S27" s="4">
+      <c r="S27" s="3">
         <v>68741.52</v>
       </c>
       <c r="T27">
-        <f>D27/S27</f>
+        <f t="shared" si="6"/>
         <v>89.615140893014868</v>
       </c>
       <c r="U27">
@@ -3721,11 +3713,11 @@
       <c r="Y27">
         <v>35</v>
       </c>
-      <c r="Z27" s="5">
+      <c r="Z27" s="4">
         <v>501650</v>
       </c>
-      <c r="AA27" s="6">
-        <f>Z27/D27</f>
+      <c r="AA27" s="5">
+        <f t="shared" si="7"/>
         <v>8.1432973593250052E-2</v>
       </c>
     </row>
@@ -3746,15 +3738,15 @@
         <v>1080577</v>
       </c>
       <c r="F28">
-        <f>D28-C28</f>
+        <f t="shared" si="0"/>
         <v>90991</v>
       </c>
       <c r="G28">
-        <f>F28/C28*100</f>
+        <f t="shared" si="1"/>
         <v>9.1501946871329505</v>
       </c>
       <c r="H28" s="2">
-        <f>(D28-E28)/E28</f>
+        <f t="shared" si="2"/>
         <v>4.4698341719285163E-3</v>
       </c>
       <c r="I28">
@@ -3764,18 +3756,18 @@
         <v>2</v>
       </c>
       <c r="K28">
-        <f>J28-I28</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L28">
         <v>3</v>
       </c>
       <c r="M28">
-        <f>J28+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N28">
-        <f>M28-L28</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O28" t="s">
@@ -3790,11 +3782,11 @@
       <c r="R28">
         <v>0</v>
       </c>
-      <c r="S28" s="4">
+      <c r="S28" s="3">
         <v>145545.79999999999</v>
       </c>
       <c r="T28">
-        <f>D28/S28</f>
+        <f t="shared" si="6"/>
         <v>7.4574944794009861</v>
       </c>
       <c r="U28">
@@ -3812,11 +3804,11 @@
       <c r="Y28">
         <v>38</v>
       </c>
-      <c r="Z28" s="5">
+      <c r="Z28" s="4">
         <v>635500</v>
       </c>
-      <c r="AA28" s="6">
-        <f>Z28/D28</f>
+      <c r="AA28" s="5">
+        <f t="shared" si="7"/>
         <v>0.58549465776432252</v>
       </c>
     </row>
@@ -3824,7 +3816,7 @@
       <c r="A29" t="s">
         <v>37</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" t="s">
         <v>85</v>
       </c>
       <c r="C29">
@@ -3837,15 +3829,15 @@
         <v>1937552</v>
       </c>
       <c r="F29">
-        <f>D29-C29</f>
+        <f t="shared" si="0"/>
         <v>131508</v>
       </c>
       <c r="G29">
-        <f>F29/C29*100</f>
+        <f t="shared" si="1"/>
         <v>7.1790700530891334</v>
       </c>
       <c r="H29" s="2">
-        <f>(D29-E29)/E29</f>
+        <f t="shared" si="2"/>
         <v>1.330596546570105E-2</v>
       </c>
       <c r="I29">
@@ -3855,37 +3847,37 @@
         <v>3</v>
       </c>
       <c r="K29">
-        <f>J29-I29</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L29">
         <v>5</v>
       </c>
       <c r="M29">
-        <f>J29+2</f>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="N29">
-        <f>M29-L29</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O29" t="s">
         <v>9</v>
       </c>
-      <c r="P29" s="3">
+      <c r="P29">
         <v>214</v>
       </c>
-      <c r="Q29" s="3">
+      <c r="Q29">
         <v>4</v>
       </c>
-      <c r="R29" s="3">
+      <c r="R29">
         <v>1</v>
       </c>
-      <c r="S29" s="4">
+      <c r="S29" s="3">
         <v>76824.17</v>
       </c>
       <c r="T29">
-        <f>D29/S29</f>
+        <f t="shared" si="6"/>
         <v>25.556188892115593</v>
       </c>
       <c r="U29">
@@ -3903,8 +3895,8 @@
       <c r="Y29">
         <v>40</v>
       </c>
-      <c r="AA29" s="6">
-        <f>Z29/D29</f>
+      <c r="AA29" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3925,15 +3917,15 @@
         <v>3138259</v>
       </c>
       <c r="F30">
-        <f>D30-C30</f>
+        <f t="shared" si="0"/>
         <v>399030</v>
       </c>
       <c r="G30">
-        <f>F30/C30*100</f>
+        <f t="shared" si="1"/>
         <v>14.72744102823027</v>
       </c>
       <c r="H30" s="2">
-        <f>(D30-E30)/E30</f>
+        <f t="shared" si="2"/>
         <v>-9.4947548943538438E-3</v>
       </c>
       <c r="I30">
@@ -3943,18 +3935,18 @@
         <v>4</v>
       </c>
       <c r="K30">
-        <f>J30-I30</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L30">
         <v>6</v>
       </c>
       <c r="M30">
-        <f>J30+2</f>
+        <f t="shared" si="8"/>
         <v>6</v>
       </c>
       <c r="N30">
-        <f>M30-L30</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O30" t="s">
@@ -3969,11 +3961,11 @@
       <c r="R30">
         <v>6</v>
       </c>
-      <c r="S30" s="4">
+      <c r="S30" s="3">
         <v>109781.18</v>
       </c>
       <c r="T30">
-        <f>D30/S30</f>
+        <f t="shared" si="6"/>
         <v>28.315071854756891</v>
       </c>
       <c r="U30">
@@ -3991,11 +3983,11 @@
       <c r="Y30">
         <v>22</v>
       </c>
-      <c r="Z30" s="5">
+      <c r="Z30" s="4">
         <v>5000000</v>
       </c>
-      <c r="AA30" s="6">
-        <f>Z30/D30</f>
+      <c r="AA30" s="5">
+        <f t="shared" si="7"/>
         <v>1.6085125055413256</v>
       </c>
     </row>
@@ -4016,15 +4008,15 @@
         <v>1366275</v>
       </c>
       <c r="F31">
-        <f>D31-C31</f>
+        <f t="shared" si="0"/>
         <v>57644</v>
       </c>
       <c r="G31">
-        <f>F31/C31*100</f>
+        <f t="shared" si="1"/>
         <v>4.3621944159613149</v>
       </c>
       <c r="H31" s="2">
-        <f>(D31-E31)/E31</f>
+        <f t="shared" si="2"/>
         <v>9.3787853836160371E-3</v>
       </c>
       <c r="I31">
@@ -4034,18 +4026,18 @@
         <v>2</v>
       </c>
       <c r="K31">
-        <f>J31-I31</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L31">
         <v>4</v>
       </c>
       <c r="M31">
-        <f>J31+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N31">
-        <f>M31-L31</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O31" t="s">
@@ -4060,11 +4052,11 @@
       <c r="R31">
         <v>1</v>
       </c>
-      <c r="S31" s="4">
+      <c r="S31" s="3">
         <v>8952.65</v>
       </c>
       <c r="T31">
-        <f>D31/S31</f>
+        <f t="shared" si="6"/>
         <v>154.0425460617806</v>
       </c>
       <c r="U31">
@@ -4082,8 +4074,8 @@
       <c r="Y31">
         <v>19</v>
       </c>
-      <c r="AA31" s="6">
-        <f>Z31/D31</f>
+      <c r="AA31" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -4104,15 +4096,15 @@
         <v>8882371</v>
       </c>
       <c r="F32">
-        <f>D32-C32</f>
+        <f t="shared" si="0"/>
         <v>486992</v>
       </c>
       <c r="G32">
-        <f>F32/C32*100</f>
+        <f t="shared" si="1"/>
         <v>5.5292869112362295</v>
       </c>
       <c r="H32" s="2">
-        <f>(D32-E32)/E32</f>
+        <f t="shared" si="2"/>
         <v>4.6397746727759967E-2</v>
       </c>
       <c r="I32">
@@ -4122,18 +4114,18 @@
         <v>12</v>
       </c>
       <c r="K32">
-        <f>J32-I32</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L32">
         <v>14</v>
       </c>
       <c r="M32">
-        <f>J32+2</f>
+        <f t="shared" si="8"/>
         <v>14</v>
       </c>
       <c r="N32">
-        <f>M32-L32</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O32" t="s">
@@ -4148,11 +4140,11 @@
       <c r="R32">
         <v>88</v>
       </c>
-      <c r="S32" s="4">
+      <c r="S32" s="3">
         <v>7354.22</v>
       </c>
       <c r="T32">
-        <f>D32/S32</f>
+        <f t="shared" si="6"/>
         <v>1263.8312424703095</v>
       </c>
       <c r="U32">
@@ -4170,11 +4162,11 @@
       <c r="Y32">
         <v>14</v>
       </c>
-      <c r="Z32" s="5">
+      <c r="Z32" s="4">
         <v>9000000</v>
       </c>
-      <c r="AA32" s="6">
-        <f>Z32/D32</f>
+      <c r="AA32" s="5">
+        <f t="shared" si="7"/>
         <v>0.96831532392353192</v>
       </c>
     </row>
@@ -4195,15 +4187,15 @@
         <v>2106319</v>
       </c>
       <c r="F33">
-        <f>D33-C33</f>
+        <f t="shared" si="0"/>
         <v>52947</v>
       </c>
       <c r="G33">
-        <f>F33/C33*100</f>
+        <f t="shared" si="1"/>
         <v>2.5612001898152785</v>
       </c>
       <c r="H33" s="2">
-        <f>(D33-E33)/E33</f>
+        <f t="shared" si="2"/>
         <v>6.5996651029592386E-3</v>
       </c>
       <c r="I33">
@@ -4213,18 +4205,18 @@
         <v>3</v>
       </c>
       <c r="K33">
-        <f>J33-I33</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L33">
         <v>5</v>
       </c>
       <c r="M33">
-        <f>J33+2</f>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="N33">
-        <f>M33-L33</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O33" t="s">
@@ -4239,11 +4231,11 @@
       <c r="R33">
         <v>1</v>
       </c>
-      <c r="S33" s="4">
+      <c r="S33" s="3">
         <v>121298.15</v>
       </c>
       <c r="T33">
-        <f>D33/S33</f>
+        <f t="shared" si="6"/>
         <v>17.479409207807375</v>
       </c>
       <c r="U33">
@@ -4261,11 +4253,11 @@
       <c r="Y33">
         <v>16</v>
       </c>
-      <c r="Z33" s="5">
+      <c r="Z33" s="4">
         <v>11500000</v>
       </c>
-      <c r="AA33" s="6">
-        <f>Z33/D33</f>
+      <c r="AA33" s="5">
+        <f t="shared" si="7"/>
         <v>5.4239654375489339</v>
       </c>
     </row>
@@ -4286,15 +4278,15 @@
         <v>19336776</v>
       </c>
       <c r="F34">
-        <f>D34-C34</f>
+        <f t="shared" ref="F34:F52" si="10">D34-C34</f>
         <v>794696</v>
       </c>
       <c r="G34">
-        <f>F34/C34*100</f>
+        <f t="shared" ref="G34:G52" si="11">F34/C34*100</f>
         <v>4.0919301242903643</v>
       </c>
       <c r="H34" s="2">
-        <f>(D34-E34)/E34</f>
+        <f t="shared" ref="H34:H52" si="12">(D34-E34)/E34</f>
         <v>4.5456129811919009E-2</v>
       </c>
       <c r="I34">
@@ -4304,37 +4296,37 @@
         <v>26</v>
       </c>
       <c r="K34">
-        <f>J34-I34</f>
+        <f t="shared" ref="K34:K52" si="13">J34-I34</f>
         <v>-1</v>
       </c>
       <c r="L34">
         <v>29</v>
       </c>
       <c r="M34">
-        <f>J34+2</f>
+        <f t="shared" si="8"/>
         <v>28</v>
       </c>
       <c r="N34">
-        <f>M34-L34</f>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="O34" t="s">
         <v>12</v>
       </c>
       <c r="P34">
-        <v>84735</v>
+        <v>133197</v>
       </c>
       <c r="Q34">
-        <v>1672</v>
+        <v>3069</v>
       </c>
       <c r="R34">
-        <v>365</v>
-      </c>
-      <c r="S34" s="4">
+        <v>666</v>
+      </c>
+      <c r="S34" s="3">
         <v>47126.400000000001</v>
       </c>
       <c r="T34">
-        <f>D34/S34</f>
+        <f t="shared" ref="T34:T52" si="14">D34/S34</f>
         <v>428.96870968289534</v>
       </c>
       <c r="U34">
@@ -4352,11 +4344,11 @@
       <c r="Y34">
         <v>7</v>
       </c>
-      <c r="Z34" s="5">
+      <c r="Z34" s="4">
         <v>20000000</v>
       </c>
-      <c r="AA34" s="6">
-        <f>Z34/D34</f>
+      <c r="AA34" s="5">
+        <f t="shared" ref="AA34:AA52" si="15">Z34/D34</f>
         <v>0.98932757927222192</v>
       </c>
     </row>
@@ -4377,15 +4369,15 @@
         <v>10600823</v>
       </c>
       <c r="F35">
-        <f>D35-C35</f>
+        <f t="shared" si="10"/>
         <v>888167</v>
       </c>
       <c r="G35">
-        <f>F35/C35*100</f>
+        <f t="shared" si="11"/>
         <v>9.2848351849159005</v>
       </c>
       <c r="H35" s="2">
-        <f>(D35-E35)/E35</f>
+        <f t="shared" si="12"/>
         <v>-1.3855056347983548E-2</v>
       </c>
       <c r="I35">
@@ -4395,18 +4387,18 @@
         <v>14</v>
       </c>
       <c r="K35">
-        <f>J35-I35</f>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="L35">
         <v>15</v>
       </c>
       <c r="M35">
-        <f>J35+2</f>
+        <f t="shared" si="8"/>
         <v>16</v>
       </c>
       <c r="N35">
-        <f>M35-L35</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O35" t="s">
@@ -4421,11 +4413,11 @@
       <c r="R35">
         <v>1</v>
       </c>
-      <c r="S35" s="4">
+      <c r="S35" s="3">
         <v>48617.91</v>
       </c>
       <c r="T35">
-        <f>D35/S35</f>
+        <f t="shared" si="14"/>
         <v>215.02257090031225</v>
       </c>
       <c r="U35">
@@ -4443,11 +4435,11 @@
       <c r="Y35">
         <v>27</v>
       </c>
-      <c r="Z35" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA35" s="6">
-        <f>Z35/D35</f>
+      <c r="Z35" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -4468,15 +4460,15 @@
         <v>765309</v>
       </c>
       <c r="F36">
-        <f>D36-C36</f>
+        <f t="shared" si="10"/>
         <v>103797</v>
       </c>
       <c r="G36">
-        <f>F36/C36*100</f>
+        <f t="shared" si="11"/>
         <v>15.356743921113175</v>
       </c>
       <c r="H36" s="2">
-        <f>(D36-E36)/E36</f>
+        <f t="shared" si="12"/>
         <v>1.8806782619830684E-2</v>
       </c>
       <c r="I36">
@@ -4486,18 +4478,18 @@
         <v>1</v>
       </c>
       <c r="K36">
-        <f>J36-I36</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L36">
         <v>3</v>
       </c>
       <c r="M36">
-        <f>J36+2</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="N36">
-        <f>M36-L36</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O36" t="s">
@@ -4512,11 +4504,11 @@
       <c r="R36">
         <v>0</v>
       </c>
-      <c r="S36" s="4">
+      <c r="S36" s="3">
         <v>69000.800000000003</v>
       </c>
       <c r="T36">
-        <f>D36/S36</f>
+        <f t="shared" si="14"/>
         <v>11.299897972197423</v>
       </c>
       <c r="U36">
@@ -4534,11 +4526,11 @@
       <c r="Y36">
         <v>49</v>
       </c>
-      <c r="Z36" s="5">
+      <c r="Z36" s="4">
         <v>1000000</v>
       </c>
-      <c r="AA36" s="6">
-        <f>Z36/D36</f>
+      <c r="AA36" s="5">
+        <f t="shared" si="15"/>
         <v>1.2825412785910515</v>
       </c>
     </row>
@@ -4559,15 +4551,15 @@
         <v>11693217</v>
       </c>
       <c r="F37">
-        <f>D37-C37</f>
+        <f t="shared" si="10"/>
         <v>240353</v>
       </c>
       <c r="G37">
-        <f>F37/C37*100</f>
+        <f t="shared" si="11"/>
         <v>2.0776514144666183</v>
       </c>
       <c r="H37" s="2">
-        <f>(D37-E37)/E37</f>
+        <f t="shared" si="12"/>
         <v>9.8887243775600854E-3</v>
       </c>
       <c r="I37">
@@ -4577,18 +4569,18 @@
         <v>15</v>
       </c>
       <c r="K37">
-        <f>J37-I37</f>
+        <f t="shared" si="13"/>
         <v>-1</v>
       </c>
       <c r="L37">
         <v>18</v>
       </c>
       <c r="M37">
-        <f>J37+2</f>
+        <f t="shared" si="8"/>
         <v>17</v>
       </c>
       <c r="N37">
-        <f>M37-L37</f>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="O37" t="s">
@@ -4603,11 +4595,11 @@
       <c r="R37">
         <v>10</v>
       </c>
-      <c r="S37" s="4">
+      <c r="S37" s="3">
         <v>40860.69</v>
       </c>
       <c r="T37">
-        <f>D37/S37</f>
+        <f t="shared" si="14"/>
         <v>289.00265756647769</v>
       </c>
       <c r="U37">
@@ -4625,11 +4617,11 @@
       <c r="Y37">
         <v>30</v>
       </c>
-      <c r="Z37" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA37" s="6">
-        <f>Z37/D37</f>
+      <c r="Z37" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -4650,15 +4642,15 @@
         <v>3980783</v>
       </c>
       <c r="F38">
-        <f>D38-C38</f>
+        <f t="shared" si="10"/>
         <v>198634</v>
       </c>
       <c r="G38">
-        <f>F38/C38*100</f>
+        <f t="shared" si="11"/>
         <v>5.2759688085841736</v>
       </c>
       <c r="H38" s="2">
-        <f>(D38-E38)/E38</f>
+        <f t="shared" si="12"/>
         <v>-4.3375888612868377E-3</v>
       </c>
       <c r="I38">
@@ -4668,18 +4660,18 @@
         <v>5</v>
       </c>
       <c r="K38">
-        <f>J38-I38</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L38">
         <v>7</v>
       </c>
       <c r="M38">
-        <f>J38+2</f>
+        <f t="shared" si="8"/>
         <v>7</v>
       </c>
       <c r="N38">
-        <f>M38-L38</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O38" t="s">
@@ -4694,11 +4686,11 @@
       <c r="R38">
         <v>5</v>
       </c>
-      <c r="S38" s="4">
+      <c r="S38" s="3">
         <v>68594.92</v>
       </c>
       <c r="T38">
-        <f>D38/S38</f>
+        <f t="shared" si="14"/>
         <v>57.781480027967085</v>
       </c>
       <c r="U38">
@@ -4716,11 +4708,11 @@
       <c r="Y38">
         <v>48</v>
       </c>
-      <c r="Z38" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA38" s="6">
-        <f>Z38/D38</f>
+      <c r="Z38" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA38" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -4741,15 +4733,15 @@
         <v>4241507</v>
       </c>
       <c r="F39">
-        <f>D39-C39</f>
+        <f t="shared" si="10"/>
         <v>392894</v>
       </c>
       <c r="G39">
-        <f>F39/C39*100</f>
+        <f t="shared" si="11"/>
         <v>10.208735318710204</v>
       </c>
       <c r="H39" s="2">
-        <f>(D39-E39)/E39</f>
+        <f t="shared" si="12"/>
         <v>-1.6503568189325161E-6</v>
       </c>
       <c r="I39">
@@ -4759,18 +4751,18 @@
         <v>6</v>
       </c>
       <c r="K39">
-        <f>J39-I39</f>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="L39">
         <v>7</v>
       </c>
       <c r="M39">
-        <f>J39+2</f>
+        <f t="shared" si="8"/>
         <v>8</v>
       </c>
       <c r="N39">
-        <f>M39-L39</f>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O39" t="s">
@@ -4785,11 +4777,11 @@
       <c r="R39">
         <v>0</v>
       </c>
-      <c r="S39" s="4">
+      <c r="S39" s="3">
         <v>95988.01</v>
       </c>
       <c r="T39">
-        <f>D39/S39</f>
+        <f t="shared" si="14"/>
         <v>44.187810540087249</v>
       </c>
       <c r="U39">
@@ -4807,11 +4799,11 @@
       <c r="Y39">
         <v>13</v>
       </c>
-      <c r="Z39" s="5">
+      <c r="Z39" s="4">
         <v>7730772</v>
       </c>
-      <c r="AA39" s="6">
-        <f>Z39/D39</f>
+      <c r="AA39" s="5">
+        <f t="shared" si="15"/>
         <v>1.8226504774254391</v>
       </c>
     </row>
@@ -4832,15 +4824,15 @@
         <v>12783254</v>
       </c>
       <c r="F40">
-        <f>D40-C40</f>
+        <f t="shared" si="10"/>
         <v>276939</v>
       </c>
       <c r="G40">
-        <f>F40/C40*100</f>
+        <f t="shared" si="11"/>
         <v>2.1746451975888319</v>
       </c>
       <c r="H40" s="2">
-        <f>(D40-E40)/E40</f>
+        <f t="shared" si="12"/>
         <v>1.7881988420162816E-2</v>
       </c>
       <c r="I40">
@@ -4850,18 +4842,18 @@
         <v>17</v>
       </c>
       <c r="K40">
-        <f>J40-I40</f>
+        <f t="shared" si="13"/>
         <v>-1</v>
       </c>
       <c r="L40">
         <v>20</v>
       </c>
       <c r="M40">
-        <f>J40+2</f>
+        <f t="shared" si="8"/>
         <v>19</v>
       </c>
       <c r="N40">
-        <f>M40-L40</f>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="O40" t="s">
@@ -4876,11 +4868,11 @@
       <c r="R40">
         <v>11</v>
       </c>
-      <c r="S40" s="4">
+      <c r="S40" s="3">
         <v>44742.7</v>
       </c>
       <c r="T40">
-        <f>D40/S40</f>
+        <f t="shared" si="14"/>
         <v>290.81490388376204</v>
       </c>
       <c r="U40">
@@ -4898,11 +4890,11 @@
       <c r="Y40">
         <v>23</v>
       </c>
-      <c r="Z40" s="5">
+      <c r="Z40" s="4">
         <v>4000000</v>
       </c>
-      <c r="AA40" s="6">
-        <f>Z40/D40</f>
+      <c r="AA40" s="5">
+        <f t="shared" si="15"/>
         <v>0.30741223150231434</v>
       </c>
     </row>
@@ -4923,15 +4915,15 @@
         <v>1057125</v>
       </c>
       <c r="F41">
-        <f>D41-C41</f>
+        <f t="shared" si="10"/>
         <v>42916</v>
       </c>
       <c r="G41">
-        <f>F41/C41*100</f>
+        <f t="shared" si="11"/>
         <v>4.0669151392991401</v>
       </c>
       <c r="H41" s="2">
-        <f>(D41-E41)/E41</f>
+        <f t="shared" si="12"/>
         <v>3.8820385479484451E-2</v>
       </c>
       <c r="I41">
@@ -4941,18 +4933,18 @@
         <v>2</v>
       </c>
       <c r="K41">
-        <f>J41-I41</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L41">
         <v>4</v>
       </c>
       <c r="M41">
-        <f>J41+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N41">
-        <f>M41-L41</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O41" t="s">
@@ -4967,11 +4959,11 @@
       <c r="R41">
         <v>1</v>
       </c>
-      <c r="S41" s="4">
+      <c r="S41" s="3">
         <v>1033.81</v>
       </c>
       <c r="T41">
-        <f>D41/S41</f>
+        <f t="shared" si="14"/>
         <v>1062.2483821978894</v>
       </c>
       <c r="U41">
@@ -4989,11 +4981,11 @@
       <c r="Y41">
         <v>8</v>
       </c>
-      <c r="Z41" s="5">
+      <c r="Z41" s="4">
         <v>500000</v>
       </c>
-      <c r="AA41" s="6">
-        <f>Z41/D41</f>
+      <c r="AA41" s="5">
+        <f t="shared" si="15"/>
         <v>0.45530581525693364</v>
       </c>
     </row>
@@ -5014,15 +5006,15 @@
         <v>5218040</v>
       </c>
       <c r="F42">
-        <f>D42-C42</f>
+        <f t="shared" si="10"/>
         <v>478737</v>
       </c>
       <c r="G42">
-        <f>F42/C42*100</f>
+        <f t="shared" si="11"/>
         <v>10.304338701779498</v>
       </c>
       <c r="H42" s="2">
-        <f>(D42-E42)/E42</f>
+        <f t="shared" si="12"/>
         <v>-1.7885642885067957E-2</v>
       </c>
       <c r="I42">
@@ -5032,18 +5024,18 @@
         <v>7</v>
       </c>
       <c r="K42">
-        <f>J42-I42</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L42">
         <v>9</v>
       </c>
       <c r="M42">
-        <f>J42+2</f>
+        <f t="shared" si="8"/>
         <v>9</v>
       </c>
       <c r="N42">
-        <f>M42-L42</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O42" t="s">
@@ -5058,11 +5050,11 @@
       <c r="R42">
         <v>2</v>
       </c>
-      <c r="S42" s="4">
+      <c r="S42" s="3">
         <v>30060.7</v>
       </c>
       <c r="T42">
-        <f>D42/S42</f>
+        <f t="shared" si="14"/>
         <v>170.47879789891786</v>
       </c>
       <c r="U42">
@@ -5080,11 +5072,11 @@
       <c r="Y42">
         <v>33</v>
       </c>
-      <c r="Z42" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA42" s="6">
-        <f>Z42/D42</f>
+      <c r="Z42" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -5105,15 +5097,15 @@
         <v>892717</v>
       </c>
       <c r="F43">
-        <f>D43-C43</f>
+        <f t="shared" si="10"/>
         <v>68009</v>
       </c>
       <c r="G43">
-        <f>F43/C43*100</f>
+        <f t="shared" si="11"/>
         <v>8.2961985261557949</v>
       </c>
       <c r="H43" s="2">
-        <f>(D43-E43)/E43</f>
+        <f t="shared" si="12"/>
         <v>-5.5415097953774826E-3</v>
       </c>
       <c r="I43">
@@ -5123,18 +5115,18 @@
         <v>1</v>
       </c>
       <c r="K43">
-        <f>J43-I43</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L43">
         <v>3</v>
       </c>
       <c r="M43">
-        <f>J43+2</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="N43">
-        <f>M43-L43</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O43" t="s">
@@ -5149,11 +5141,11 @@
       <c r="R43">
         <v>1</v>
       </c>
-      <c r="S43" s="4">
+      <c r="S43" s="3">
         <v>75811</v>
       </c>
       <c r="T43">
-        <f>D43/S43</f>
+        <f t="shared" si="14"/>
         <v>11.710305892284762</v>
       </c>
       <c r="U43">
@@ -5171,11 +5163,11 @@
       <c r="Y43">
         <v>45</v>
       </c>
-      <c r="Z43" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA43" s="6">
-        <f>Z43/D43</f>
+      <c r="Z43" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA43" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -5196,15 +5188,15 @@
         <v>6886834</v>
       </c>
       <c r="F44">
-        <f>D44-C44</f>
+        <f t="shared" si="10"/>
         <v>541466</v>
       </c>
       <c r="G44">
-        <f>F44/C44*100</f>
+        <f t="shared" si="11"/>
         <v>8.4930101196295578</v>
       </c>
       <c r="H44" s="2">
-        <f>(D44-E44)/E44</f>
+        <f t="shared" si="12"/>
         <v>4.3652859935349106E-3</v>
       </c>
       <c r="I44">
@@ -5214,18 +5206,18 @@
         <v>9</v>
       </c>
       <c r="K44">
-        <f>J44-I44</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L44">
         <v>11</v>
       </c>
       <c r="M44">
-        <f>J44+2</f>
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
       <c r="N44">
-        <f>M44-L44</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O44" t="s">
@@ -5240,11 +5232,11 @@
       <c r="R44">
         <v>0</v>
       </c>
-      <c r="S44" s="4">
+      <c r="S44" s="3">
         <v>41234.9</v>
       </c>
       <c r="T44">
-        <f>D44/S44</f>
+        <f t="shared" si="14"/>
         <v>167.74375589609772</v>
       </c>
       <c r="U44">
@@ -5262,11 +5254,11 @@
       <c r="Y44">
         <v>42</v>
       </c>
-      <c r="Z44" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA44" s="6">
-        <f>Z44/D44</f>
+      <c r="Z44" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA44" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -5287,15 +5279,15 @@
         <v>29360759</v>
       </c>
       <c r="F45">
-        <f>D45-C45</f>
+        <f t="shared" si="10"/>
         <v>3914872</v>
       </c>
       <c r="G45">
-        <f>F45/C45*100</f>
+        <f t="shared" si="11"/>
         <v>15.493142467407338</v>
       </c>
       <c r="H45" s="2">
-        <f>(D45-E45)/E45</f>
+        <f t="shared" si="12"/>
         <v>-6.0444282111371851E-3</v>
       </c>
       <c r="I45">
@@ -5305,18 +5297,18 @@
         <v>38</v>
       </c>
       <c r="K45">
-        <f>J45-I45</f>
+        <f t="shared" si="13"/>
         <v>2</v>
       </c>
       <c r="L45">
         <v>38</v>
       </c>
       <c r="M45">
-        <f>J45+2</f>
+        <f t="shared" si="8"/>
         <v>40</v>
       </c>
       <c r="N45">
-        <f>M45-L45</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
       <c r="O45" t="s">
@@ -5331,11 +5323,11 @@
       <c r="R45">
         <v>21</v>
       </c>
-      <c r="S45" s="4">
+      <c r="S45" s="3">
         <v>261231.71</v>
       </c>
       <c r="T45">
-        <f>D45/S45</f>
+        <f t="shared" si="14"/>
         <v>111.71419426837576</v>
       </c>
       <c r="U45">
@@ -5353,11 +5345,11 @@
       <c r="Y45">
         <v>29</v>
       </c>
-      <c r="Z45" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA45" s="6">
-        <f>Z45/D45</f>
+      <c r="Z45" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA45" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -5378,15 +5370,15 @@
         <v>3249879</v>
       </c>
       <c r="F46">
-        <f>D46-C46</f>
+        <f t="shared" si="10"/>
         <v>504487</v>
       </c>
       <c r="G46">
-        <f>F46/C46*100</f>
+        <f t="shared" si="11"/>
         <v>18.207498651094554</v>
       </c>
       <c r="H46" s="2">
-        <f>(D46-E46)/E46</f>
+        <f t="shared" si="12"/>
         <v>7.8073675973782406E-3</v>
       </c>
       <c r="I46">
@@ -5396,18 +5388,18 @@
         <v>4</v>
       </c>
       <c r="K46">
-        <f>J46-I46</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L46">
         <v>6</v>
       </c>
       <c r="M46">
-        <f>J46+2</f>
+        <f t="shared" si="8"/>
         <v>6</v>
       </c>
       <c r="N46">
-        <f>M46-L46</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O46" t="s">
@@ -5422,11 +5414,11 @@
       <c r="R46">
         <v>2</v>
       </c>
-      <c r="S46" s="4">
+      <c r="S46" s="3">
         <v>82169.62</v>
       </c>
       <c r="T46">
-        <f>D46/S46</f>
+        <f t="shared" si="14"/>
         <v>39.859646424067684</v>
       </c>
       <c r="U46">
@@ -5444,11 +5436,11 @@
       <c r="Y46">
         <v>41</v>
       </c>
-      <c r="Z46" s="5">
+      <c r="Z46" s="4">
         <v>1000000</v>
       </c>
-      <c r="AA46" s="6">
-        <f>Z46/D46</f>
+      <c r="AA46" s="5">
+        <f t="shared" si="15"/>
         <v>0.30532001812379628</v>
       </c>
     </row>
@@ -5457,7 +5449,7 @@
         <v>55</v>
       </c>
       <c r="B47" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C47">
         <v>630337</v>
@@ -5469,15 +5461,15 @@
         <v>623347</v>
       </c>
       <c r="F47">
-        <f>D47-C47</f>
+        <f t="shared" si="10"/>
         <v>13166</v>
       </c>
       <c r="G47">
-        <f>F47/C47*100</f>
+        <f t="shared" si="11"/>
         <v>2.0887239682899783</v>
       </c>
       <c r="H47" s="2">
-        <f>(D47-E47)/E47</f>
+        <f t="shared" si="12"/>
         <v>3.233511992517811E-2</v>
       </c>
       <c r="I47">
@@ -5487,37 +5479,37 @@
         <v>1</v>
       </c>
       <c r="K47">
-        <f>J47-I47</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L47">
         <v>3</v>
       </c>
       <c r="M47">
-        <f>J47+2</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="N47">
-        <f>M47-L47</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O47" t="s">
         <v>12</v>
       </c>
       <c r="P47">
-        <v>1706</v>
+        <v>321</v>
       </c>
       <c r="Q47">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="R47">
-        <v>7</v>
-      </c>
-      <c r="S47" s="4">
+        <v>3</v>
+      </c>
+      <c r="S47" s="3">
         <v>9216.66</v>
       </c>
       <c r="T47">
-        <f>D47/S47</f>
+        <f t="shared" si="14"/>
         <v>69.819544173268838</v>
       </c>
       <c r="U47">
@@ -5535,11 +5527,11 @@
       <c r="Y47">
         <v>2</v>
       </c>
-      <c r="Z47" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA47" s="6">
-        <f>Z47/D47</f>
+      <c r="Z47" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA47" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
@@ -5548,7 +5540,7 @@
         <v>56</v>
       </c>
       <c r="B48" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C48">
         <v>8037736</v>
@@ -5560,15 +5552,15 @@
         <v>8590563</v>
       </c>
       <c r="F48">
-        <f>D48-C48</f>
+        <f t="shared" si="10"/>
         <v>616806</v>
       </c>
       <c r="G48">
-        <f>F48/C48*100</f>
+        <f t="shared" si="11"/>
         <v>7.6738773206783604</v>
       </c>
       <c r="H48" s="2">
-        <f>(D48-E48)/E48</f>
+        <f t="shared" si="12"/>
         <v>7.4475910368156312E-3</v>
       </c>
       <c r="I48">
@@ -5578,37 +5570,37 @@
         <v>11</v>
       </c>
       <c r="K48">
-        <f>J48-I48</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L48">
         <v>13</v>
       </c>
       <c r="M48">
-        <f>J48+2</f>
+        <f t="shared" si="8"/>
         <v>13</v>
       </c>
       <c r="N48">
-        <f>M48-L48</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O48" t="s">
         <v>12</v>
       </c>
       <c r="P48">
-        <v>321</v>
+        <v>1706</v>
       </c>
       <c r="Q48">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="R48">
-        <v>3</v>
-      </c>
-      <c r="S48" s="4">
+        <v>7</v>
+      </c>
+      <c r="S48" s="3">
         <v>39490.089999999997</v>
       </c>
       <c r="T48">
-        <f>D48/S48</f>
+        <f t="shared" si="14"/>
         <v>219.15731263210594</v>
       </c>
       <c r="U48">
@@ -5626,11 +5618,11 @@
       <c r="Y48">
         <v>17</v>
       </c>
-      <c r="Z48" s="5">
+      <c r="Z48" s="4">
         <v>1500000</v>
       </c>
-      <c r="AA48" s="6">
-        <f>Z48/D48</f>
+      <c r="AA48" s="5">
+        <f t="shared" si="15"/>
         <v>0.17331939691320464</v>
       </c>
     </row>
@@ -5651,15 +5643,15 @@
         <v>7693612</v>
       </c>
       <c r="F49">
-        <f>D49-C49</f>
+        <f t="shared" si="10"/>
         <v>962577</v>
       </c>
       <c r="G49">
-        <f>F49/C49*100</f>
+        <f t="shared" si="11"/>
         <v>14.25328602657429</v>
       </c>
       <c r="H49" s="2">
-        <f>(D49-E49)/E49</f>
+        <f t="shared" si="12"/>
         <v>2.9029277795656967E-3</v>
       </c>
       <c r="I49">
@@ -5669,18 +5661,18 @@
         <v>10</v>
       </c>
       <c r="K49">
-        <f>J49-I49</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L49">
         <v>12</v>
       </c>
       <c r="M49">
-        <f>J49+2</f>
+        <f t="shared" si="8"/>
         <v>12</v>
       </c>
       <c r="N49">
-        <f>M49-L49</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O49" t="s">
@@ -5695,11 +5687,11 @@
       <c r="R49">
         <v>51</v>
       </c>
-      <c r="S49" s="4">
+      <c r="S49" s="3">
         <v>66455.520000000004</v>
       </c>
       <c r="T49">
-        <f>D49/S49</f>
+        <f t="shared" si="14"/>
         <v>116.10692384921522</v>
       </c>
       <c r="U49">
@@ -5717,11 +5709,11 @@
       <c r="Y49">
         <v>10</v>
       </c>
-      <c r="Z49" s="5">
+      <c r="Z49" s="4">
         <v>15464000</v>
       </c>
-      <c r="AA49" s="6">
-        <f>Z49/D49</f>
+      <c r="AA49" s="5">
+        <f t="shared" si="15"/>
         <v>2.0041612525541264</v>
       </c>
     </row>
@@ -5742,15 +5734,15 @@
         <v>1784787</v>
       </c>
       <c r="F50">
-        <f>D50-C50</f>
+        <f t="shared" si="10"/>
         <v>-64770</v>
       </c>
       <c r="G50">
-        <f>F50/C50*100</f>
+        <f t="shared" si="11"/>
         <v>-3.4826044525934035</v>
       </c>
       <c r="H50" s="2">
-        <f>(D50-E50)/E50</f>
+        <f t="shared" si="12"/>
         <v>5.7474645433880905E-3</v>
       </c>
       <c r="I50">
@@ -5760,18 +5752,18 @@
         <v>2</v>
       </c>
       <c r="K50">
-        <f>J50-I50</f>
+        <f t="shared" si="13"/>
         <v>-1</v>
       </c>
       <c r="L50">
         <v>5</v>
       </c>
       <c r="M50">
-        <f>J50+2</f>
+        <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="N50">
-        <f>M50-L50</f>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="O50" t="s">
@@ -5786,11 +5778,11 @@
       <c r="R50">
         <v>1</v>
       </c>
-      <c r="S50" s="4">
+      <c r="S50" s="3">
         <v>24038.21</v>
       </c>
       <c r="T50">
-        <f>D50/S50</f>
+        <f t="shared" si="14"/>
         <v>74.674653395573131</v>
       </c>
       <c r="U50">
@@ -5808,11 +5800,11 @@
       <c r="Y50">
         <v>50</v>
       </c>
-      <c r="Z50" s="5">
+      <c r="Z50" s="4">
         <v>1000000</v>
       </c>
-      <c r="AA50" s="6">
-        <f>Z50/D50</f>
+      <c r="AA50" s="5">
+        <f t="shared" si="15"/>
         <v>0.55708909804489581</v>
       </c>
     </row>
@@ -5833,15 +5825,15 @@
         <v>5832655</v>
       </c>
       <c r="F51">
-        <f>D51-C51</f>
+        <f t="shared" si="10"/>
         <v>199243</v>
       </c>
       <c r="G51">
-        <f>F51/C51*100</f>
+        <f t="shared" si="11"/>
         <v>3.4965770072461098</v>
       </c>
       <c r="H51" s="2">
-        <f>(D51-E51)/E51</f>
+        <f t="shared" si="12"/>
         <v>1.1112949420118283E-2</v>
       </c>
       <c r="I51">
@@ -5851,18 +5843,18 @@
         <v>8</v>
       </c>
       <c r="K51">
-        <f>J51-I51</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L51">
         <v>10</v>
       </c>
       <c r="M51">
-        <f>J51+2</f>
+        <f t="shared" si="8"/>
         <v>10</v>
       </c>
       <c r="N51">
-        <f>M51-L51</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O51" t="s">
@@ -5877,11 +5869,11 @@
       <c r="R51">
         <v>8</v>
       </c>
-      <c r="S51" s="4">
+      <c r="S51" s="3">
         <v>54157.8</v>
       </c>
       <c r="T51">
-        <f>D51/S51</f>
+        <f t="shared" si="14"/>
         <v>108.8942497664233</v>
       </c>
       <c r="U51">
@@ -5899,11 +5891,11 @@
       <c r="Y51">
         <v>24</v>
       </c>
-      <c r="Z51" s="5">
+      <c r="Z51" s="4">
         <v>1000000</v>
       </c>
-      <c r="AA51" s="6">
-        <f>Z51/D51</f>
+      <c r="AA51" s="5">
+        <f t="shared" si="15"/>
         <v>0.16956415061162636</v>
       </c>
     </row>
@@ -5924,15 +5916,15 @@
         <v>582328</v>
       </c>
       <c r="F52">
-        <f>D52-C52</f>
+        <f t="shared" si="10"/>
         <v>9419</v>
       </c>
       <c r="G52">
-        <f>F52/C52*100</f>
+        <f t="shared" si="11"/>
         <v>1.6573992609537216</v>
       </c>
       <c r="H52" s="2">
-        <f>(D52-E52)/E52</f>
+        <f t="shared" si="12"/>
         <v>-7.914783421027324E-3</v>
       </c>
       <c r="I52">
@@ -5942,18 +5934,18 @@
         <v>1</v>
       </c>
       <c r="K52">
-        <f>J52-I52</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L52">
         <v>3</v>
       </c>
       <c r="M52">
-        <f>J52+2</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="N52">
-        <f>M52-L52</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O52" t="s">
@@ -5968,11 +5960,11 @@
       <c r="R52">
         <v>0</v>
       </c>
-      <c r="S52" s="4">
+      <c r="S52" s="3">
         <v>97093.14</v>
       </c>
       <c r="T52">
-        <f>D52/S52</f>
+        <f t="shared" si="14"/>
         <v>5.9501526060440524</v>
       </c>
       <c r="U52">
@@ -5990,11 +5982,11 @@
       <c r="Y52">
         <v>51</v>
       </c>
-      <c r="Z52" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA52" s="6">
-        <f>Z52/D52</f>
+      <c r="Z52" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="5">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>